<commit_message>
feat: liệt kê tổng thầu turnkey theo khung nguồn trong market-research, bản 0.6.12
Danh sách nhà thầu trước đây dựng từ tìm kiếm web chung nên lệch về đại lý
trung gian, và bị chặn ở 3-5 đơn vị do dùng chung quota báo cáo.

- SKILL.md §6 mới: taxonomy Tổng thầu turnkey / Cấp 1 chuyên ngành /
  Trung gian-Đại lý / Chưa xác định; 10 khung nguồn F1-F10 (đấu thầu,
  chứng chỉ năng lực HĐXD, điện lực, ĐKKD, Sở Xây dựng, dự án ngược,
  snowball, ngành lân cận, hiệp hội, trang đại lý hãng); bộ mã ngành
  VSIC dương/âm; điều kiện bằng chứng turnkey; thang điểm và Nhóm A/B/C;
  quy tắc bão hòa và ngân sách riêng.
- Bỏ loại trừ theo từ khóa "đại lý"/"phân phối": tổng thầu vừa thi công
  vừa phân phối thiết bị là bình thường, chỉ loại khi thiếu bằng chứng
  tự thi công.
- §12 audit E và §13 gate độ phủ cho danh sách nhà thầu.
- Workbook: thêm sheet Bảng 3B (18 cột, khóa mã số thuế, sổ loại trừ,
  khối độ phủ F1-F10); Bảng 3 dòng 28 rút thành tóm tắt; dòng 55 chỉ
  chọn từ Nhóm A.
</commit_message>
<xml_diff>
--- a/skills/market-research/assets/khung-bao-cao-thi-truong.xlsx
+++ b/skills/market-research/assets/khung-bao-cao-thi-truong.xlsx
@@ -7,7 +7,8 @@
   </bookViews>
   <sheets>
     <sheet name="Khung báo cáo thị trường mẫu" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="00 - Hướng dẫn" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Bảng 3B - Danh sách nhà thầu" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="00 - Hướng dẫn" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -151,7 +152,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -281,11 +282,69 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -392,6 +451,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1768,7 +1845,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Liệt kê tối thiểu 3–5 đơn vị có bằng chứng hoạt động tại thị trường; tên pháp lý, website và liên hệ công khai. Nếu ít hơn, nêu phạm vi đã tìm.</t>
+          <t>Liệt kê ĐẦY ĐỦ tại sheet 'Bảng 3B - Danh sách nhà thầu' (mỗi dòng một công ty, khóa theo mã số thuế); ô này chỉ tóm tắt: tổng số đơn vị, số Tổng thầu turnkey, số thuộc Nhóm A, và 3–5 đơn vị dẫn đầu kèm tên pháp lý, website, liên hệ công khai. Danh sách phải dựng theo khung nguồn (§6.2 SKILL.md) và dừng theo quy tắc bão hòa — 3–5 là mức sàn cho ô tóm tắt này, không phải mục tiêu của danh sách.</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1785,7 +1862,7 @@
       <c r="E28" s="2" t="inlineStr">
         <is>
           <t>Dự án tham chiếu phải có địa điểm, năm, phạm vi công việc và nguồn. Phân biệt thông tin tự công bố với nguồn độc lập/chủ đầu tư.
-Vai trò chuỗi cung ứng: Thi công trực tiếp (Cấp 1) / Trung gian-Đại lý (Cấp 2) / Chưa xác định, kèm bằng chứng. Mã ngành thuộc nhóm thương mại/phân phối, hoặc mô tả công khai chỉ dùng ngôn ngữ đại lý/phân phối/ủy quyền không kèm bằng chứng tự thi công, phải ghi Cấp 2 và loại khỏi danh sách 'Nhà thầu phù hợp sơ bộ'.</t>
+Vai trò chuỗi cung ứng ghi tại Bảng 3B: Tổng thầu turnkey / Cấp 1 chuyên ngành / Trung gian-Đại lý (Cấp 2) / Chưa xác định. Chỉ Tổng thầu turnkey mới vào danh sách 'Nhà thầu phù hợp sơ bộ'. Turnkey bắt buộc có ≥1 bằng chứng độc lập; hồ sơ năng lực tự công bố không đủ. Không loại đơn vị chỉ vì website có chữ đại lý/phân phối — nhiều tổng thầu vừa thi công vừa phân phối thiết bị; chỉ loại khi thiếu bằng chứng tự thi công.</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -2942,7 +3019,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Chỉ chọn từ đơn vị đã phân loại Cấp 1 (thi công trực tiếp) ở Bảng 3. Nếu không đủ Cấp 1, được đưa Cấp 2/Chưa xác định nhưng phải ghi rõ và nêu lý do. Xếp hạng ưu tiên: có báo chí/nguồn độc lập xác nhận dự án &gt; chỉ có dự án tham chiếu tự công bố &gt; 1 nguồn duy nhất. Đưa danh sách 1–3 đơn vị kèm bằng chứng và nội dung còn thiếu. Không coi là lựa chọn cuối trước khi kiểm tra pháp lý, tham chiếu dự án và nhận hồ sơ/báo giá.</t>
+          <t>Chỉ chọn từ đơn vị đã phân loại 'Tổng thầu turnkey' và thuộc Nhóm A ở Bảng 3B. Nếu không đủ, được đưa nhóm thấp hơn nhưng phải ghi rõ nhóm, điểm và lý do. Xếp hạng: dự án trúng thầu/chủ đầu tư xác nhận &gt; báo chí độc lập &gt; tự công bố. Đưa 1–3 đơn vị kèm bằng chứng và nội dung còn thiếu. Không coi là lựa chọn cuối trước khi kiểm tra pháp lý, tham chiếu dự án và nhận hồ sơ/báo giá.</t>
         </is>
       </c>
       <c r="C55" s="4" t="n"/>
@@ -26284,6 +26361,1506 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:R83"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="38" t="inlineStr">
+        <is>
+          <t>BẢNG 3B — DANH SÁCH NHÀ THẦU (mỗi dòng một công ty, khóa theo mã số thuế)</t>
+        </is>
+      </c>
+      <c r="B1" s="39" t="n"/>
+      <c r="C1" s="39" t="n"/>
+      <c r="D1" s="39" t="n"/>
+      <c r="E1" s="39" t="n"/>
+      <c r="F1" s="39" t="n"/>
+      <c r="G1" s="39" t="n"/>
+      <c r="H1" s="39" t="n"/>
+      <c r="I1" s="39" t="n"/>
+      <c r="J1" s="39" t="n"/>
+      <c r="K1" s="39" t="n"/>
+      <c r="L1" s="39" t="n"/>
+      <c r="M1" s="39" t="n"/>
+      <c r="N1" s="39" t="n"/>
+      <c r="O1" s="39" t="n"/>
+      <c r="P1" s="39" t="n"/>
+      <c r="Q1" s="39" t="n"/>
+      <c r="R1" s="40" t="n"/>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="41" t="inlineStr">
+        <is>
+          <t>Mục tiêu mặc định: TỔNG THẦU TURNKEY (EPC/EC) — đơn vị tự thi công và lo trọn gói: thiết kế, vật tư/thiết bị, thi công, xin phép, thử nghiệm/nghiệm thu. Liệt kê theo khung nguồn (§6.2 SKILL.md), không bắt đầu bằng tìm kiếm web chung. Dừng theo quy tắc bão hòa, không dừng ở 3–5 đơn vị.</t>
+        </is>
+      </c>
+      <c r="B2" s="39" t="n"/>
+      <c r="C2" s="39" t="n"/>
+      <c r="D2" s="39" t="n"/>
+      <c r="E2" s="39" t="n"/>
+      <c r="F2" s="39" t="n"/>
+      <c r="G2" s="39" t="n"/>
+      <c r="H2" s="39" t="n"/>
+      <c r="I2" s="39" t="n"/>
+      <c r="J2" s="39" t="n"/>
+      <c r="K2" s="39" t="n"/>
+      <c r="L2" s="39" t="n"/>
+      <c r="M2" s="39" t="n"/>
+      <c r="N2" s="39" t="n"/>
+      <c r="O2" s="39" t="n"/>
+      <c r="P2" s="39" t="n"/>
+      <c r="Q2" s="39" t="n"/>
+      <c r="R2" s="40" t="n"/>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="42" t="inlineStr">
+        <is>
+          <t>MST</t>
+        </is>
+      </c>
+      <c r="B3" s="42" t="inlineStr">
+        <is>
+          <t>Tên pháp lý</t>
+        </is>
+      </c>
+      <c r="C3" s="42" t="inlineStr">
+        <is>
+          <t>Tên thương mại / thương hiệu</t>
+        </is>
+      </c>
+      <c r="D3" s="42" t="inlineStr">
+        <is>
+          <t>Địa bàn hoạt động</t>
+        </is>
+      </c>
+      <c r="E3" s="42" t="inlineStr">
+        <is>
+          <t>Mã ngành chính</t>
+        </is>
+      </c>
+      <c r="F3" s="42" t="inlineStr">
+        <is>
+          <t>Ngày cấp ĐKKD</t>
+        </is>
+      </c>
+      <c r="G3" s="42" t="inlineStr">
+        <is>
+          <t>Chứng chỉ năng lực HĐXD</t>
+        </is>
+      </c>
+      <c r="H3" s="42" t="inlineStr">
+        <is>
+          <t>Vai trò chuỗi cung ứng</t>
+        </is>
+      </c>
+      <c r="I3" s="42" t="inlineStr">
+        <is>
+          <t>Dự án tham chiếu</t>
+        </is>
+      </c>
+      <c r="J3" s="42" t="inlineStr">
+        <is>
+          <t>Báo chí độc lập</t>
+        </is>
+      </c>
+      <c r="K3" s="42" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="L3" s="42" t="inlineStr">
+        <is>
+          <t>LinkedIn / mạng xã hội</t>
+        </is>
+      </c>
+      <c r="M3" s="42" t="inlineStr">
+        <is>
+          <t>Điểm</t>
+        </is>
+      </c>
+      <c r="N3" s="42" t="inlineStr">
+        <is>
+          <t>Nhóm</t>
+        </is>
+      </c>
+      <c r="O3" s="42" t="inlineStr">
+        <is>
+          <t>Khung phát hiện</t>
+        </is>
+      </c>
+      <c r="P3" s="42" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="Q3" s="42" t="inlineStr">
+        <is>
+          <t>Liên hệ công khai</t>
+        </is>
+      </c>
+      <c r="R3" s="42" t="inlineStr">
+        <is>
+          <t>Ghi chú / nội dung còn thiếu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="120" customHeight="1">
+      <c r="A4" s="41" t="inlineStr">
+        <is>
+          <t>Mã số thuế — khóa định danh duy nhất. Một công ty = một dòng, dù xuất hiện ở nhiều khung tìm kiếm.</t>
+        </is>
+      </c>
+      <c r="B4" s="41" t="inlineStr">
+        <is>
+          <t>Tên trên đăng ký kinh doanh, kèm URL tra cứu.</t>
+        </is>
+      </c>
+      <c r="C4" s="41" t="inlineStr">
+        <is>
+          <t>Tên hay dùng trên website, báo chí, biển hiệu. Để trống nếu trùng tên pháp lý.</t>
+        </is>
+      </c>
+      <c r="D4" s="41" t="inlineStr">
+        <is>
+          <t>Trụ sở và các tỉnh/thành có bằng chứng đã thi công.</t>
+        </is>
+      </c>
+      <c r="E4" s="41" t="inlineStr">
+        <is>
+          <t>Mã VSIC + tên ngành + nguồn (cổng ĐKKD). Ghi thêm mã ngành phụ liên quan thi công/thiết kế nếu có.</t>
+        </is>
+      </c>
+      <c r="F4" s="41" t="inlineStr">
+        <is>
+          <t>dd/mm/yyyy + nguồn. Không suy đoán từ năm ghi trên website.</t>
+        </is>
+      </c>
+      <c r="G4" s="41" t="inlineStr">
+        <is>
+          <t>Số chứng chỉ | hạng I/II/III | lĩnh vực | hiệu lực | nguồn (nangluchdxd.gov.vn hoặc Sở Xây dựng). Không tìm thấy: Chưa xác minh.</t>
+        </is>
+      </c>
+      <c r="H4" s="41" t="inlineStr">
+        <is>
+          <t>Tổng thầu turnkey / Cấp 1 chuyên ngành / Trung gian-Đại lý (Cấp 2) / Chưa xác định. Bắt buộc kèm bằng chứng. Turnkey phải có ≥1 bằng chứng độc lập (gói EC/EPC trúng thầu, chứng chỉ cả thiết kế lẫn thi công, hoặc dự án trọn gói do chủ đầu tư/báo chí mô tả).</t>
+        </is>
+      </c>
+      <c r="I4" s="41" t="inlineStr">
+        <is>
+          <t>Tên dự án | chủ đầu tư | địa điểm | năm | phạm vi công việc | nguồn. Ghi rõ nguồn là kết quả đấu thầu / chủ đầu tư / báo chí / tự công bố.</t>
+        </is>
+      </c>
+      <c r="J4" s="41" t="inlineStr">
+        <is>
+          <t>Tiêu đề bài + ngày + URL. Bài PR tự đăng phải ghi rõ là tự công bố.</t>
+        </is>
+      </c>
+      <c r="K4" s="41" t="inlineStr">
+        <is>
+          <t>URL + đã mở trong lần chạy này hay chưa. Ghi ngắn nội dung mô tả năng lực.</t>
+        </is>
+      </c>
+      <c r="L4" s="41" t="inlineStr">
+        <is>
+          <t>URL + mô tả công ty có nêu thi công/xây lắp/tổng thầu/EPC hay không.</t>
+        </is>
+      </c>
+      <c r="M4" s="41" t="inlineStr">
+        <is>
+          <t>Tổng điểm theo thang §6.5 của SKILL.md. Ghi điểm từng tiêu chí ở cột Ghi chú nếu cần.</t>
+        </is>
+      </c>
+      <c r="N4" s="41" t="inlineStr">
+        <is>
+          <t>A: ≥8 điểm + ≥1 dự án nguồn độc lập + vai trò Tổng thầu turnkey. B: 5–7, hoặc ≥8 nhưng chưa đủ bằng chứng turnkey. C: &lt;5 hoặc Chưa xác định.</t>
+        </is>
+      </c>
+      <c r="O4" s="41" t="inlineStr">
+        <is>
+          <t>Khung nào tìm ra đơn vị này (F1 đấu thầu, F2 chứng chỉ năng lực, F3 điện lực, F4 ĐKKD, F5 Sở Xây dựng, F6 dự án ngược, F7 snowball, F8 ngành lân cận, F9 hiệp hội, F10 trang đại lý hãng).</t>
+        </is>
+      </c>
+      <c r="P4" s="41" t="inlineStr">
+        <is>
+          <t>Đã xác minh / Ước tính / Chưa xác minh / Không áp dụng — theo sheet 00 - Hướng dẫn.</t>
+        </is>
+      </c>
+      <c r="Q4" s="41" t="inlineStr">
+        <is>
+          <t>Điện thoại, email, địa chỉ văn phòng lấy từ nguồn công khai. Không suy đoán.</t>
+        </is>
+      </c>
+      <c r="R4" s="41" t="inlineStr">
+        <is>
+          <t>Điểm từng tiêu chí, mâu thuẫn giữa các nguồn, và dữ liệu cần đơn vị nào xác nhận.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="41" t="n"/>
+      <c r="B5" s="41" t="n"/>
+      <c r="C5" s="41" t="n"/>
+      <c r="D5" s="41" t="n"/>
+      <c r="E5" s="41" t="n"/>
+      <c r="F5" s="41" t="n"/>
+      <c r="G5" s="41" t="n"/>
+      <c r="H5" s="41" t="n"/>
+      <c r="I5" s="41" t="n"/>
+      <c r="J5" s="41" t="n"/>
+      <c r="K5" s="41" t="n"/>
+      <c r="L5" s="41" t="n"/>
+      <c r="M5" s="41" t="n"/>
+      <c r="N5" s="41" t="n"/>
+      <c r="O5" s="41" t="n"/>
+      <c r="P5" s="41" t="n"/>
+      <c r="Q5" s="41" t="n"/>
+      <c r="R5" s="41" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="43" t="n"/>
+      <c r="B6" s="41" t="n"/>
+      <c r="C6" s="41" t="n"/>
+      <c r="D6" s="41" t="n"/>
+      <c r="E6" s="41" t="n"/>
+      <c r="F6" s="41" t="n"/>
+      <c r="G6" s="41" t="n"/>
+      <c r="H6" s="41" t="n"/>
+      <c r="I6" s="41" t="n"/>
+      <c r="J6" s="41" t="n"/>
+      <c r="K6" s="41" t="n"/>
+      <c r="L6" s="41" t="n"/>
+      <c r="M6" s="41" t="n"/>
+      <c r="N6" s="41" t="n"/>
+      <c r="O6" s="41" t="n"/>
+      <c r="P6" s="41" t="n"/>
+      <c r="Q6" s="41" t="n"/>
+      <c r="R6" s="41" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="44" t="n"/>
+      <c r="B7" s="44" t="n"/>
+      <c r="C7" s="44" t="n"/>
+      <c r="D7" s="44" t="n"/>
+      <c r="E7" s="44" t="n"/>
+      <c r="F7" s="41" t="n"/>
+      <c r="G7" s="41" t="n"/>
+      <c r="H7" s="41" t="n"/>
+      <c r="I7" s="41" t="n"/>
+      <c r="J7" s="41" t="n"/>
+      <c r="K7" s="41" t="n"/>
+      <c r="L7" s="41" t="n"/>
+      <c r="M7" s="41" t="n"/>
+      <c r="N7" s="41" t="n"/>
+      <c r="O7" s="41" t="n"/>
+      <c r="P7" s="41" t="n"/>
+      <c r="Q7" s="41" t="n"/>
+      <c r="R7" s="41" t="n"/>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="41" t="n"/>
+      <c r="B8" s="41" t="n"/>
+      <c r="C8" s="41" t="n"/>
+      <c r="D8" s="41" t="n"/>
+      <c r="E8" s="41" t="n"/>
+      <c r="F8" s="41" t="n"/>
+      <c r="G8" s="41" t="n"/>
+      <c r="H8" s="41" t="n"/>
+      <c r="I8" s="41" t="n"/>
+      <c r="J8" s="41" t="n"/>
+      <c r="K8" s="41" t="n"/>
+      <c r="L8" s="41" t="n"/>
+      <c r="M8" s="41" t="n"/>
+      <c r="N8" s="41" t="n"/>
+      <c r="O8" s="41" t="n"/>
+      <c r="P8" s="41" t="n"/>
+      <c r="Q8" s="41" t="n"/>
+      <c r="R8" s="41" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="41" t="n"/>
+      <c r="B9" s="41" t="n"/>
+      <c r="C9" s="41" t="n"/>
+      <c r="D9" s="41" t="n"/>
+      <c r="E9" s="41" t="n"/>
+      <c r="F9" s="41" t="n"/>
+      <c r="G9" s="41" t="n"/>
+      <c r="H9" s="41" t="n"/>
+      <c r="I9" s="41" t="n"/>
+      <c r="J9" s="41" t="n"/>
+      <c r="K9" s="41" t="n"/>
+      <c r="L9" s="41" t="n"/>
+      <c r="M9" s="41" t="n"/>
+      <c r="N9" s="41" t="n"/>
+      <c r="O9" s="41" t="n"/>
+      <c r="P9" s="41" t="n"/>
+      <c r="Q9" s="41" t="n"/>
+      <c r="R9" s="41" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="43" t="n"/>
+      <c r="B10" s="41" t="n"/>
+      <c r="C10" s="41" t="n"/>
+      <c r="D10" s="41" t="n"/>
+      <c r="E10" s="41" t="n"/>
+      <c r="F10" s="41" t="n"/>
+      <c r="G10" s="41" t="n"/>
+      <c r="H10" s="41" t="n"/>
+      <c r="I10" s="41" t="n"/>
+      <c r="J10" s="41" t="n"/>
+      <c r="K10" s="41" t="n"/>
+      <c r="L10" s="41" t="n"/>
+      <c r="M10" s="41" t="n"/>
+      <c r="N10" s="41" t="n"/>
+      <c r="O10" s="41" t="n"/>
+      <c r="P10" s="41" t="n"/>
+      <c r="Q10" s="41" t="n"/>
+      <c r="R10" s="41" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="44" t="n"/>
+      <c r="B11" s="44" t="n"/>
+      <c r="C11" s="44" t="n"/>
+      <c r="D11" s="44" t="n"/>
+      <c r="E11" s="44" t="n"/>
+      <c r="F11" s="41" t="n"/>
+      <c r="G11" s="41" t="n"/>
+      <c r="H11" s="41" t="n"/>
+      <c r="I11" s="41" t="n"/>
+      <c r="J11" s="41" t="n"/>
+      <c r="K11" s="41" t="n"/>
+      <c r="L11" s="41" t="n"/>
+      <c r="M11" s="41" t="n"/>
+      <c r="N11" s="41" t="n"/>
+      <c r="O11" s="41" t="n"/>
+      <c r="P11" s="41" t="n"/>
+      <c r="Q11" s="41" t="n"/>
+      <c r="R11" s="41" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="41" t="n"/>
+      <c r="B12" s="41" t="n"/>
+      <c r="C12" s="41" t="n"/>
+      <c r="D12" s="41" t="n"/>
+      <c r="E12" s="41" t="n"/>
+      <c r="F12" s="41" t="n"/>
+      <c r="G12" s="41" t="n"/>
+      <c r="H12" s="41" t="n"/>
+      <c r="I12" s="41" t="n"/>
+      <c r="J12" s="41" t="n"/>
+      <c r="K12" s="41" t="n"/>
+      <c r="L12" s="41" t="n"/>
+      <c r="M12" s="41" t="n"/>
+      <c r="N12" s="41" t="n"/>
+      <c r="O12" s="41" t="n"/>
+      <c r="P12" s="41" t="n"/>
+      <c r="Q12" s="41" t="n"/>
+      <c r="R12" s="41" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="41" t="n"/>
+      <c r="B13" s="41" t="n"/>
+      <c r="C13" s="41" t="n"/>
+      <c r="D13" s="41" t="n"/>
+      <c r="E13" s="41" t="n"/>
+      <c r="F13" s="41" t="n"/>
+      <c r="G13" s="41" t="n"/>
+      <c r="H13" s="41" t="n"/>
+      <c r="I13" s="41" t="n"/>
+      <c r="J13" s="41" t="n"/>
+      <c r="K13" s="41" t="n"/>
+      <c r="L13" s="41" t="n"/>
+      <c r="M13" s="41" t="n"/>
+      <c r="N13" s="41" t="n"/>
+      <c r="O13" s="41" t="n"/>
+      <c r="P13" s="41" t="n"/>
+      <c r="Q13" s="41" t="n"/>
+      <c r="R13" s="41" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="41" t="n"/>
+      <c r="B14" s="41" t="n"/>
+      <c r="C14" s="41" t="n"/>
+      <c r="D14" s="41" t="n"/>
+      <c r="E14" s="41" t="n"/>
+      <c r="F14" s="41" t="n"/>
+      <c r="G14" s="41" t="n"/>
+      <c r="H14" s="41" t="n"/>
+      <c r="I14" s="41" t="n"/>
+      <c r="J14" s="41" t="n"/>
+      <c r="K14" s="41" t="n"/>
+      <c r="L14" s="41" t="n"/>
+      <c r="M14" s="41" t="n"/>
+      <c r="N14" s="41" t="n"/>
+      <c r="O14" s="41" t="n"/>
+      <c r="P14" s="41" t="n"/>
+      <c r="Q14" s="41" t="n"/>
+      <c r="R14" s="41" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="41" t="n"/>
+      <c r="B15" s="41" t="n"/>
+      <c r="C15" s="41" t="n"/>
+      <c r="D15" s="41" t="n"/>
+      <c r="E15" s="41" t="n"/>
+      <c r="F15" s="41" t="n"/>
+      <c r="G15" s="41" t="n"/>
+      <c r="H15" s="41" t="n"/>
+      <c r="I15" s="41" t="n"/>
+      <c r="J15" s="41" t="n"/>
+      <c r="K15" s="41" t="n"/>
+      <c r="L15" s="41" t="n"/>
+      <c r="M15" s="41" t="n"/>
+      <c r="N15" s="41" t="n"/>
+      <c r="O15" s="41" t="n"/>
+      <c r="P15" s="41" t="n"/>
+      <c r="Q15" s="41" t="n"/>
+      <c r="R15" s="41" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="41" t="n"/>
+      <c r="B16" s="41" t="n"/>
+      <c r="C16" s="41" t="n"/>
+      <c r="D16" s="41" t="n"/>
+      <c r="E16" s="41" t="n"/>
+      <c r="F16" s="41" t="n"/>
+      <c r="G16" s="41" t="n"/>
+      <c r="H16" s="41" t="n"/>
+      <c r="I16" s="41" t="n"/>
+      <c r="J16" s="41" t="n"/>
+      <c r="K16" s="41" t="n"/>
+      <c r="L16" s="41" t="n"/>
+      <c r="M16" s="41" t="n"/>
+      <c r="N16" s="41" t="n"/>
+      <c r="O16" s="41" t="n"/>
+      <c r="P16" s="41" t="n"/>
+      <c r="Q16" s="41" t="n"/>
+      <c r="R16" s="41" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="41" t="n"/>
+      <c r="B17" s="41" t="n"/>
+      <c r="C17" s="41" t="n"/>
+      <c r="D17" s="41" t="n"/>
+      <c r="E17" s="41" t="n"/>
+      <c r="F17" s="41" t="n"/>
+      <c r="G17" s="41" t="n"/>
+      <c r="H17" s="41" t="n"/>
+      <c r="I17" s="41" t="n"/>
+      <c r="J17" s="41" t="n"/>
+      <c r="K17" s="41" t="n"/>
+      <c r="L17" s="41" t="n"/>
+      <c r="M17" s="41" t="n"/>
+      <c r="N17" s="41" t="n"/>
+      <c r="O17" s="41" t="n"/>
+      <c r="P17" s="41" t="n"/>
+      <c r="Q17" s="41" t="n"/>
+      <c r="R17" s="41" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="41" t="n"/>
+      <c r="B18" s="41" t="n"/>
+      <c r="C18" s="41" t="n"/>
+      <c r="D18" s="41" t="n"/>
+      <c r="E18" s="41" t="n"/>
+      <c r="F18" s="41" t="n"/>
+      <c r="G18" s="41" t="n"/>
+      <c r="H18" s="41" t="n"/>
+      <c r="I18" s="41" t="n"/>
+      <c r="J18" s="41" t="n"/>
+      <c r="K18" s="41" t="n"/>
+      <c r="L18" s="41" t="n"/>
+      <c r="M18" s="41" t="n"/>
+      <c r="N18" s="41" t="n"/>
+      <c r="O18" s="41" t="n"/>
+      <c r="P18" s="41" t="n"/>
+      <c r="Q18" s="41" t="n"/>
+      <c r="R18" s="41" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="41" t="n"/>
+      <c r="B19" s="41" t="n"/>
+      <c r="C19" s="41" t="n"/>
+      <c r="D19" s="41" t="n"/>
+      <c r="E19" s="41" t="n"/>
+      <c r="F19" s="41" t="n"/>
+      <c r="G19" s="41" t="n"/>
+      <c r="H19" s="41" t="n"/>
+      <c r="I19" s="41" t="n"/>
+      <c r="J19" s="41" t="n"/>
+      <c r="K19" s="41" t="n"/>
+      <c r="L19" s="41" t="n"/>
+      <c r="M19" s="41" t="n"/>
+      <c r="N19" s="41" t="n"/>
+      <c r="O19" s="41" t="n"/>
+      <c r="P19" s="41" t="n"/>
+      <c r="Q19" s="41" t="n"/>
+      <c r="R19" s="41" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="41" t="n"/>
+      <c r="B20" s="41" t="n"/>
+      <c r="C20" s="41" t="n"/>
+      <c r="D20" s="41" t="n"/>
+      <c r="E20" s="41" t="n"/>
+      <c r="F20" s="41" t="n"/>
+      <c r="G20" s="41" t="n"/>
+      <c r="H20" s="41" t="n"/>
+      <c r="I20" s="41" t="n"/>
+      <c r="J20" s="41" t="n"/>
+      <c r="K20" s="41" t="n"/>
+      <c r="L20" s="41" t="n"/>
+      <c r="M20" s="41" t="n"/>
+      <c r="N20" s="41" t="n"/>
+      <c r="O20" s="41" t="n"/>
+      <c r="P20" s="41" t="n"/>
+      <c r="Q20" s="41" t="n"/>
+      <c r="R20" s="41" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="41" t="n"/>
+      <c r="B21" s="41" t="n"/>
+      <c r="C21" s="41" t="n"/>
+      <c r="D21" s="41" t="n"/>
+      <c r="E21" s="41" t="n"/>
+      <c r="F21" s="41" t="n"/>
+      <c r="G21" s="41" t="n"/>
+      <c r="H21" s="41" t="n"/>
+      <c r="I21" s="41" t="n"/>
+      <c r="J21" s="41" t="n"/>
+      <c r="K21" s="41" t="n"/>
+      <c r="L21" s="41" t="n"/>
+      <c r="M21" s="41" t="n"/>
+      <c r="N21" s="41" t="n"/>
+      <c r="O21" s="41" t="n"/>
+      <c r="P21" s="41" t="n"/>
+      <c r="Q21" s="41" t="n"/>
+      <c r="R21" s="41" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="44" t="n"/>
+      <c r="B22" s="41" t="n"/>
+      <c r="C22" s="41" t="n"/>
+      <c r="D22" s="41" t="n"/>
+      <c r="E22" s="41" t="n"/>
+      <c r="F22" s="41" t="n"/>
+      <c r="G22" s="41" t="n"/>
+      <c r="H22" s="41" t="n"/>
+      <c r="I22" s="41" t="n"/>
+      <c r="J22" s="41" t="n"/>
+      <c r="K22" s="41" t="n"/>
+      <c r="L22" s="41" t="n"/>
+      <c r="M22" s="41" t="n"/>
+      <c r="N22" s="41" t="n"/>
+      <c r="O22" s="41" t="n"/>
+      <c r="P22" s="41" t="n"/>
+      <c r="Q22" s="41" t="n"/>
+      <c r="R22" s="41" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="44" t="n"/>
+      <c r="B23" s="41" t="n"/>
+      <c r="C23" s="41" t="n"/>
+      <c r="D23" s="41" t="n"/>
+      <c r="E23" s="41" t="n"/>
+      <c r="F23" s="41" t="n"/>
+      <c r="G23" s="41" t="n"/>
+      <c r="H23" s="41" t="n"/>
+      <c r="I23" s="41" t="n"/>
+      <c r="J23" s="41" t="n"/>
+      <c r="K23" s="41" t="n"/>
+      <c r="L23" s="41" t="n"/>
+      <c r="M23" s="41" t="n"/>
+      <c r="N23" s="41" t="n"/>
+      <c r="O23" s="41" t="n"/>
+      <c r="P23" s="41" t="n"/>
+      <c r="Q23" s="41" t="n"/>
+      <c r="R23" s="41" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="41" t="n"/>
+      <c r="B24" s="41" t="n"/>
+      <c r="C24" s="41" t="n"/>
+      <c r="D24" s="41" t="n"/>
+      <c r="E24" s="41" t="n"/>
+      <c r="F24" s="41" t="n"/>
+      <c r="G24" s="41" t="n"/>
+      <c r="H24" s="41" t="n"/>
+      <c r="I24" s="41" t="n"/>
+      <c r="J24" s="41" t="n"/>
+      <c r="K24" s="41" t="n"/>
+      <c r="L24" s="41" t="n"/>
+      <c r="M24" s="41" t="n"/>
+      <c r="N24" s="41" t="n"/>
+      <c r="O24" s="41" t="n"/>
+      <c r="P24" s="41" t="n"/>
+      <c r="Q24" s="41" t="n"/>
+      <c r="R24" s="41" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="41" t="n"/>
+      <c r="B25" s="41" t="n"/>
+      <c r="C25" s="41" t="n"/>
+      <c r="D25" s="41" t="n"/>
+      <c r="E25" s="41" t="n"/>
+      <c r="F25" s="41" t="n"/>
+      <c r="G25" s="41" t="n"/>
+      <c r="H25" s="41" t="n"/>
+      <c r="I25" s="41" t="n"/>
+      <c r="J25" s="41" t="n"/>
+      <c r="K25" s="41" t="n"/>
+      <c r="L25" s="41" t="n"/>
+      <c r="M25" s="41" t="n"/>
+      <c r="N25" s="41" t="n"/>
+      <c r="O25" s="41" t="n"/>
+      <c r="P25" s="41" t="n"/>
+      <c r="Q25" s="41" t="n"/>
+      <c r="R25" s="41" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="41" t="n"/>
+      <c r="B26" s="41" t="n"/>
+      <c r="C26" s="41" t="n"/>
+      <c r="D26" s="41" t="n"/>
+      <c r="E26" s="41" t="n"/>
+      <c r="F26" s="41" t="n"/>
+      <c r="G26" s="41" t="n"/>
+      <c r="H26" s="41" t="n"/>
+      <c r="I26" s="41" t="n"/>
+      <c r="J26" s="41" t="n"/>
+      <c r="K26" s="41" t="n"/>
+      <c r="L26" s="41" t="n"/>
+      <c r="M26" s="41" t="n"/>
+      <c r="N26" s="41" t="n"/>
+      <c r="O26" s="41" t="n"/>
+      <c r="P26" s="41" t="n"/>
+      <c r="Q26" s="41" t="n"/>
+      <c r="R26" s="41" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="41" t="n"/>
+      <c r="B27" s="41" t="n"/>
+      <c r="C27" s="41" t="n"/>
+      <c r="D27" s="41" t="n"/>
+      <c r="E27" s="41" t="n"/>
+      <c r="F27" s="41" t="n"/>
+      <c r="G27" s="41" t="n"/>
+      <c r="H27" s="41" t="n"/>
+      <c r="I27" s="41" t="n"/>
+      <c r="J27" s="41" t="n"/>
+      <c r="K27" s="41" t="n"/>
+      <c r="L27" s="41" t="n"/>
+      <c r="M27" s="41" t="n"/>
+      <c r="N27" s="41" t="n"/>
+      <c r="O27" s="41" t="n"/>
+      <c r="P27" s="41" t="n"/>
+      <c r="Q27" s="41" t="n"/>
+      <c r="R27" s="41" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="41" t="n"/>
+      <c r="B28" s="41" t="n"/>
+      <c r="C28" s="41" t="n"/>
+      <c r="D28" s="41" t="n"/>
+      <c r="E28" s="41" t="n"/>
+      <c r="F28" s="41" t="n"/>
+      <c r="G28" s="41" t="n"/>
+      <c r="H28" s="41" t="n"/>
+      <c r="I28" s="41" t="n"/>
+      <c r="J28" s="41" t="n"/>
+      <c r="K28" s="41" t="n"/>
+      <c r="L28" s="41" t="n"/>
+      <c r="M28" s="41" t="n"/>
+      <c r="N28" s="41" t="n"/>
+      <c r="O28" s="41" t="n"/>
+      <c r="P28" s="41" t="n"/>
+      <c r="Q28" s="41" t="n"/>
+      <c r="R28" s="41" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="41" t="n"/>
+      <c r="B29" s="41" t="n"/>
+      <c r="C29" s="41" t="n"/>
+      <c r="D29" s="41" t="n"/>
+      <c r="E29" s="41" t="n"/>
+      <c r="F29" s="41" t="n"/>
+      <c r="G29" s="41" t="n"/>
+      <c r="H29" s="41" t="n"/>
+      <c r="I29" s="41" t="n"/>
+      <c r="J29" s="41" t="n"/>
+      <c r="K29" s="41" t="n"/>
+      <c r="L29" s="41" t="n"/>
+      <c r="M29" s="41" t="n"/>
+      <c r="N29" s="41" t="n"/>
+      <c r="O29" s="41" t="n"/>
+      <c r="P29" s="41" t="n"/>
+      <c r="Q29" s="41" t="n"/>
+      <c r="R29" s="41" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="41" t="n"/>
+      <c r="B30" s="41" t="n"/>
+      <c r="C30" s="41" t="n"/>
+      <c r="D30" s="41" t="n"/>
+      <c r="E30" s="41" t="n"/>
+      <c r="F30" s="41" t="n"/>
+      <c r="G30" s="41" t="n"/>
+      <c r="H30" s="41" t="n"/>
+      <c r="I30" s="41" t="n"/>
+      <c r="J30" s="41" t="n"/>
+      <c r="K30" s="41" t="n"/>
+      <c r="L30" s="41" t="n"/>
+      <c r="M30" s="41" t="n"/>
+      <c r="N30" s="41" t="n"/>
+      <c r="O30" s="41" t="n"/>
+      <c r="P30" s="41" t="n"/>
+      <c r="Q30" s="41" t="n"/>
+      <c r="R30" s="41" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="41" t="n"/>
+      <c r="B31" s="41" t="n"/>
+      <c r="C31" s="41" t="n"/>
+      <c r="D31" s="41" t="n"/>
+      <c r="E31" s="41" t="n"/>
+      <c r="F31" s="41" t="n"/>
+      <c r="G31" s="41" t="n"/>
+      <c r="H31" s="41" t="n"/>
+      <c r="I31" s="41" t="n"/>
+      <c r="J31" s="41" t="n"/>
+      <c r="K31" s="41" t="n"/>
+      <c r="L31" s="41" t="n"/>
+      <c r="M31" s="41" t="n"/>
+      <c r="N31" s="41" t="n"/>
+      <c r="O31" s="41" t="n"/>
+      <c r="P31" s="41" t="n"/>
+      <c r="Q31" s="41" t="n"/>
+      <c r="R31" s="41" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="41" t="n"/>
+      <c r="B32" s="41" t="n"/>
+      <c r="C32" s="41" t="n"/>
+      <c r="D32" s="41" t="n"/>
+      <c r="E32" s="41" t="n"/>
+      <c r="F32" s="41" t="n"/>
+      <c r="G32" s="41" t="n"/>
+      <c r="H32" s="41" t="n"/>
+      <c r="I32" s="41" t="n"/>
+      <c r="J32" s="41" t="n"/>
+      <c r="K32" s="41" t="n"/>
+      <c r="L32" s="41" t="n"/>
+      <c r="M32" s="41" t="n"/>
+      <c r="N32" s="41" t="n"/>
+      <c r="O32" s="41" t="n"/>
+      <c r="P32" s="41" t="n"/>
+      <c r="Q32" s="41" t="n"/>
+      <c r="R32" s="41" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="41" t="n"/>
+      <c r="B33" s="41" t="n"/>
+      <c r="C33" s="41" t="n"/>
+      <c r="D33" s="41" t="n"/>
+      <c r="E33" s="41" t="n"/>
+      <c r="F33" s="41" t="n"/>
+      <c r="G33" s="41" t="n"/>
+      <c r="H33" s="41" t="n"/>
+      <c r="I33" s="41" t="n"/>
+      <c r="J33" s="41" t="n"/>
+      <c r="K33" s="41" t="n"/>
+      <c r="L33" s="41" t="n"/>
+      <c r="M33" s="41" t="n"/>
+      <c r="N33" s="41" t="n"/>
+      <c r="O33" s="41" t="n"/>
+      <c r="P33" s="41" t="n"/>
+      <c r="Q33" s="41" t="n"/>
+      <c r="R33" s="41" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="41" t="n"/>
+      <c r="B34" s="41" t="n"/>
+      <c r="C34" s="41" t="n"/>
+      <c r="D34" s="41" t="n"/>
+      <c r="E34" s="41" t="n"/>
+      <c r="F34" s="41" t="n"/>
+      <c r="G34" s="41" t="n"/>
+      <c r="H34" s="41" t="n"/>
+      <c r="I34" s="41" t="n"/>
+      <c r="J34" s="41" t="n"/>
+      <c r="K34" s="41" t="n"/>
+      <c r="L34" s="41" t="n"/>
+      <c r="M34" s="41" t="n"/>
+      <c r="N34" s="41" t="n"/>
+      <c r="O34" s="41" t="n"/>
+      <c r="P34" s="41" t="n"/>
+      <c r="Q34" s="41" t="n"/>
+      <c r="R34" s="41" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="41" t="n"/>
+      <c r="B35" s="41" t="n"/>
+      <c r="C35" s="41" t="n"/>
+      <c r="D35" s="41" t="n"/>
+      <c r="E35" s="41" t="n"/>
+      <c r="F35" s="41" t="n"/>
+      <c r="G35" s="41" t="n"/>
+      <c r="H35" s="41" t="n"/>
+      <c r="I35" s="41" t="n"/>
+      <c r="J35" s="41" t="n"/>
+      <c r="K35" s="41" t="n"/>
+      <c r="L35" s="41" t="n"/>
+      <c r="M35" s="41" t="n"/>
+      <c r="N35" s="41" t="n"/>
+      <c r="O35" s="41" t="n"/>
+      <c r="P35" s="41" t="n"/>
+      <c r="Q35" s="41" t="n"/>
+      <c r="R35" s="41" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="41" t="n"/>
+      <c r="B36" s="41" t="n"/>
+      <c r="C36" s="41" t="n"/>
+      <c r="D36" s="41" t="n"/>
+      <c r="E36" s="41" t="n"/>
+      <c r="F36" s="41" t="n"/>
+      <c r="G36" s="41" t="n"/>
+      <c r="H36" s="41" t="n"/>
+      <c r="I36" s="41" t="n"/>
+      <c r="J36" s="41" t="n"/>
+      <c r="K36" s="41" t="n"/>
+      <c r="L36" s="41" t="n"/>
+      <c r="M36" s="41" t="n"/>
+      <c r="N36" s="41" t="n"/>
+      <c r="O36" s="41" t="n"/>
+      <c r="P36" s="41" t="n"/>
+      <c r="Q36" s="41" t="n"/>
+      <c r="R36" s="41" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="41" t="n"/>
+      <c r="B37" s="41" t="n"/>
+      <c r="C37" s="41" t="n"/>
+      <c r="D37" s="41" t="n"/>
+      <c r="E37" s="41" t="n"/>
+      <c r="F37" s="41" t="n"/>
+      <c r="G37" s="41" t="n"/>
+      <c r="H37" s="41" t="n"/>
+      <c r="I37" s="41" t="n"/>
+      <c r="J37" s="41" t="n"/>
+      <c r="K37" s="41" t="n"/>
+      <c r="L37" s="41" t="n"/>
+      <c r="M37" s="41" t="n"/>
+      <c r="N37" s="41" t="n"/>
+      <c r="O37" s="41" t="n"/>
+      <c r="P37" s="41" t="n"/>
+      <c r="Q37" s="41" t="n"/>
+      <c r="R37" s="41" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="41" t="n"/>
+      <c r="B38" s="41" t="n"/>
+      <c r="C38" s="41" t="n"/>
+      <c r="D38" s="41" t="n"/>
+      <c r="E38" s="41" t="n"/>
+      <c r="F38" s="41" t="n"/>
+      <c r="G38" s="41" t="n"/>
+      <c r="H38" s="41" t="n"/>
+      <c r="I38" s="41" t="n"/>
+      <c r="J38" s="41" t="n"/>
+      <c r="K38" s="41" t="n"/>
+      <c r="L38" s="41" t="n"/>
+      <c r="M38" s="41" t="n"/>
+      <c r="N38" s="41" t="n"/>
+      <c r="O38" s="41" t="n"/>
+      <c r="P38" s="41" t="n"/>
+      <c r="Q38" s="41" t="n"/>
+      <c r="R38" s="41" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="41" t="n"/>
+      <c r="B39" s="41" t="n"/>
+      <c r="C39" s="41" t="n"/>
+      <c r="D39" s="41" t="n"/>
+      <c r="E39" s="41" t="n"/>
+      <c r="F39" s="41" t="n"/>
+      <c r="G39" s="41" t="n"/>
+      <c r="H39" s="41" t="n"/>
+      <c r="I39" s="41" t="n"/>
+      <c r="J39" s="41" t="n"/>
+      <c r="K39" s="41" t="n"/>
+      <c r="L39" s="41" t="n"/>
+      <c r="M39" s="41" t="n"/>
+      <c r="N39" s="41" t="n"/>
+      <c r="O39" s="41" t="n"/>
+      <c r="P39" s="41" t="n"/>
+      <c r="Q39" s="41" t="n"/>
+      <c r="R39" s="41" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="41" t="n"/>
+      <c r="B40" s="41" t="n"/>
+      <c r="C40" s="41" t="n"/>
+      <c r="D40" s="41" t="n"/>
+      <c r="E40" s="41" t="n"/>
+      <c r="F40" s="41" t="n"/>
+      <c r="G40" s="41" t="n"/>
+      <c r="H40" s="41" t="n"/>
+      <c r="I40" s="41" t="n"/>
+      <c r="J40" s="41" t="n"/>
+      <c r="K40" s="41" t="n"/>
+      <c r="L40" s="41" t="n"/>
+      <c r="M40" s="41" t="n"/>
+      <c r="N40" s="41" t="n"/>
+      <c r="O40" s="41" t="n"/>
+      <c r="P40" s="41" t="n"/>
+      <c r="Q40" s="41" t="n"/>
+      <c r="R40" s="41" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="41" t="n"/>
+      <c r="B41" s="41" t="n"/>
+      <c r="C41" s="41" t="n"/>
+      <c r="D41" s="41" t="n"/>
+      <c r="E41" s="41" t="n"/>
+      <c r="F41" s="41" t="n"/>
+      <c r="G41" s="41" t="n"/>
+      <c r="H41" s="41" t="n"/>
+      <c r="I41" s="41" t="n"/>
+      <c r="J41" s="41" t="n"/>
+      <c r="K41" s="41" t="n"/>
+      <c r="L41" s="41" t="n"/>
+      <c r="M41" s="41" t="n"/>
+      <c r="N41" s="41" t="n"/>
+      <c r="O41" s="41" t="n"/>
+      <c r="P41" s="41" t="n"/>
+      <c r="Q41" s="41" t="n"/>
+      <c r="R41" s="41" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="41" t="n"/>
+      <c r="B42" s="41" t="n"/>
+      <c r="C42" s="41" t="n"/>
+      <c r="D42" s="41" t="n"/>
+      <c r="E42" s="41" t="n"/>
+      <c r="F42" s="41" t="n"/>
+      <c r="G42" s="41" t="n"/>
+      <c r="H42" s="41" t="n"/>
+      <c r="I42" s="41" t="n"/>
+      <c r="J42" s="41" t="n"/>
+      <c r="K42" s="41" t="n"/>
+      <c r="L42" s="41" t="n"/>
+      <c r="M42" s="41" t="n"/>
+      <c r="N42" s="41" t="n"/>
+      <c r="O42" s="41" t="n"/>
+      <c r="P42" s="41" t="n"/>
+      <c r="Q42" s="41" t="n"/>
+      <c r="R42" s="41" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="41" t="n"/>
+      <c r="B43" s="41" t="n"/>
+      <c r="C43" s="41" t="n"/>
+      <c r="D43" s="41" t="n"/>
+      <c r="E43" s="41" t="n"/>
+      <c r="F43" s="41" t="n"/>
+      <c r="G43" s="41" t="n"/>
+      <c r="H43" s="41" t="n"/>
+      <c r="I43" s="41" t="n"/>
+      <c r="J43" s="41" t="n"/>
+      <c r="K43" s="41" t="n"/>
+      <c r="L43" s="41" t="n"/>
+      <c r="M43" s="41" t="n"/>
+      <c r="N43" s="41" t="n"/>
+      <c r="O43" s="41" t="n"/>
+      <c r="P43" s="41" t="n"/>
+      <c r="Q43" s="41" t="n"/>
+      <c r="R43" s="41" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="41" t="n"/>
+      <c r="B44" s="41" t="n"/>
+      <c r="C44" s="41" t="n"/>
+      <c r="D44" s="41" t="n"/>
+      <c r="E44" s="41" t="n"/>
+      <c r="F44" s="41" t="n"/>
+      <c r="G44" s="41" t="n"/>
+      <c r="H44" s="41" t="n"/>
+      <c r="I44" s="41" t="n"/>
+      <c r="J44" s="41" t="n"/>
+      <c r="K44" s="41" t="n"/>
+      <c r="L44" s="41" t="n"/>
+      <c r="M44" s="41" t="n"/>
+      <c r="N44" s="41" t="n"/>
+      <c r="O44" s="41" t="n"/>
+      <c r="P44" s="41" t="n"/>
+      <c r="Q44" s="41" t="n"/>
+      <c r="R44" s="41" t="n"/>
+    </row>
+    <row r="46" ht="24" customHeight="1">
+      <c r="A46" s="38" t="inlineStr">
+        <is>
+          <t>SỔ LOẠI TRỪ — mọi ứng viên bị loại phải có một dòng ở đây. Bỏ ứng viên trong im lặng là lỗi độ phủ.</t>
+        </is>
+      </c>
+      <c r="B46" s="39" t="n"/>
+      <c r="C46" s="39" t="n"/>
+      <c r="D46" s="39" t="n"/>
+      <c r="E46" s="39" t="n"/>
+      <c r="F46" s="39" t="n"/>
+      <c r="G46" s="39" t="n"/>
+      <c r="H46" s="39" t="n"/>
+      <c r="I46" s="39" t="n"/>
+      <c r="J46" s="39" t="n"/>
+      <c r="K46" s="39" t="n"/>
+      <c r="L46" s="39" t="n"/>
+      <c r="M46" s="39" t="n"/>
+      <c r="N46" s="39" t="n"/>
+      <c r="O46" s="39" t="n"/>
+      <c r="P46" s="39" t="n"/>
+      <c r="Q46" s="39" t="n"/>
+      <c r="R46" s="40" t="n"/>
+    </row>
+    <row r="47" ht="44" customHeight="1">
+      <c r="A47" s="42" t="inlineStr">
+        <is>
+          <t>MST</t>
+        </is>
+      </c>
+      <c r="B47" s="42" t="inlineStr">
+        <is>
+          <t>Tên đơn vị</t>
+        </is>
+      </c>
+      <c r="C47" s="42" t="inlineStr">
+        <is>
+          <t>Lý do loại (cụ thể, ví dụ: mã ngành chính 4659 bán buôn, không có bằng chứng tự thi công)</t>
+        </is>
+      </c>
+      <c r="D47" s="42" t="inlineStr">
+        <is>
+          <t>Bằng chứng / nguồn</t>
+        </is>
+      </c>
+      <c r="E47" s="42" t="inlineStr">
+        <is>
+          <t>Khung phát hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="41" t="n"/>
+      <c r="B48" s="41" t="n"/>
+      <c r="C48" s="41" t="n"/>
+      <c r="D48" s="41" t="n"/>
+      <c r="E48" s="41" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="41" t="n"/>
+      <c r="B49" s="41" t="n"/>
+      <c r="C49" s="41" t="n"/>
+      <c r="D49" s="41" t="n"/>
+      <c r="E49" s="41" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="41" t="n"/>
+      <c r="B50" s="41" t="n"/>
+      <c r="C50" s="41" t="n"/>
+      <c r="D50" s="41" t="n"/>
+      <c r="E50" s="41" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="41" t="n"/>
+      <c r="B51" s="41" t="n"/>
+      <c r="C51" s="41" t="n"/>
+      <c r="D51" s="41" t="n"/>
+      <c r="E51" s="41" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="41" t="n"/>
+      <c r="B52" s="41" t="n"/>
+      <c r="C52" s="41" t="n"/>
+      <c r="D52" s="41" t="n"/>
+      <c r="E52" s="41" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="41" t="n"/>
+      <c r="B53" s="41" t="n"/>
+      <c r="C53" s="41" t="n"/>
+      <c r="D53" s="41" t="n"/>
+      <c r="E53" s="41" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="41" t="n"/>
+      <c r="B54" s="41" t="n"/>
+      <c r="C54" s="41" t="n"/>
+      <c r="D54" s="41" t="n"/>
+      <c r="E54" s="41" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="41" t="n"/>
+      <c r="B55" s="41" t="n"/>
+      <c r="C55" s="41" t="n"/>
+      <c r="D55" s="41" t="n"/>
+      <c r="E55" s="41" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="41" t="n"/>
+      <c r="B56" s="41" t="n"/>
+      <c r="C56" s="41" t="n"/>
+      <c r="D56" s="41" t="n"/>
+      <c r="E56" s="41" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="41" t="n"/>
+      <c r="B57" s="41" t="n"/>
+      <c r="C57" s="41" t="n"/>
+      <c r="D57" s="41" t="n"/>
+      <c r="E57" s="41" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="41" t="n"/>
+      <c r="B58" s="41" t="n"/>
+      <c r="C58" s="41" t="n"/>
+      <c r="D58" s="41" t="n"/>
+      <c r="E58" s="41" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="41" t="n"/>
+      <c r="B59" s="41" t="n"/>
+      <c r="C59" s="41" t="n"/>
+      <c r="D59" s="41" t="n"/>
+      <c r="E59" s="41" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="41" t="n"/>
+      <c r="B60" s="41" t="n"/>
+      <c r="C60" s="41" t="n"/>
+      <c r="D60" s="41" t="n"/>
+      <c r="E60" s="41" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="41" t="n"/>
+      <c r="B61" s="41" t="n"/>
+      <c r="C61" s="41" t="n"/>
+      <c r="D61" s="41" t="n"/>
+      <c r="E61" s="41" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="41" t="n"/>
+      <c r="B62" s="41" t="n"/>
+      <c r="C62" s="41" t="n"/>
+      <c r="D62" s="41" t="n"/>
+      <c r="E62" s="41" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="41" t="n"/>
+      <c r="B63" s="41" t="n"/>
+      <c r="C63" s="41" t="n"/>
+      <c r="D63" s="41" t="n"/>
+      <c r="E63" s="41" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="41" t="n"/>
+      <c r="B64" s="41" t="n"/>
+      <c r="C64" s="41" t="n"/>
+      <c r="D64" s="41" t="n"/>
+      <c r="E64" s="41" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="41" t="n"/>
+      <c r="B65" s="41" t="n"/>
+      <c r="C65" s="41" t="n"/>
+      <c r="D65" s="41" t="n"/>
+      <c r="E65" s="41" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="41" t="n"/>
+      <c r="B66" s="41" t="n"/>
+      <c r="C66" s="41" t="n"/>
+      <c r="D66" s="41" t="n"/>
+      <c r="E66" s="41" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="41" t="n"/>
+      <c r="B67" s="41" t="n"/>
+      <c r="C67" s="41" t="n"/>
+      <c r="D67" s="41" t="n"/>
+      <c r="E67" s="41" t="n"/>
+    </row>
+    <row r="69" ht="24" customHeight="1">
+      <c r="A69" s="38" t="inlineStr">
+        <is>
+          <t>ĐỘ PHỦ TÌM KIẾM — bằng chứng cho tuyên bố "danh sách đầy đủ"</t>
+        </is>
+      </c>
+      <c r="B69" s="39" t="n"/>
+      <c r="C69" s="39" t="n"/>
+      <c r="D69" s="39" t="n"/>
+      <c r="E69" s="39" t="n"/>
+      <c r="F69" s="39" t="n"/>
+      <c r="G69" s="39" t="n"/>
+      <c r="H69" s="39" t="n"/>
+      <c r="I69" s="39" t="n"/>
+      <c r="J69" s="39" t="n"/>
+      <c r="K69" s="39" t="n"/>
+      <c r="L69" s="39" t="n"/>
+      <c r="M69" s="39" t="n"/>
+      <c r="N69" s="39" t="n"/>
+      <c r="O69" s="39" t="n"/>
+      <c r="P69" s="39" t="n"/>
+      <c r="Q69" s="39" t="n"/>
+      <c r="R69" s="40" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="42" t="inlineStr">
+        <is>
+          <t>Khung</t>
+        </is>
+      </c>
+      <c r="B70" s="42" t="inlineStr">
+        <is>
+          <t>Nguồn đã dùng (URL)</t>
+        </is>
+      </c>
+      <c r="C70" s="42" t="inlineStr">
+        <is>
+          <t>Đã quét?</t>
+        </is>
+      </c>
+      <c r="D70" s="42" t="inlineStr">
+        <is>
+          <t>Số MST mới</t>
+        </is>
+      </c>
+      <c r="E70" s="42" t="inlineStr">
+        <is>
+          <t>Ghi chú / lý do bỏ qua</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="41" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B71" s="41" t="inlineStr">
+        <is>
+          <t>Kết quả lựa chọn nhà thầu (muasamcong.mpi.gov.vn) — gói EC/EPC, thiết kế và thi công, chìa khóa trao tay</t>
+        </is>
+      </c>
+      <c r="C71" s="45" t="n"/>
+      <c r="D71" s="45" t="n"/>
+      <c r="E71" s="45" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="41" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="B72" s="41" t="inlineStr">
+        <is>
+          <t>Chứng chỉ năng lực hoạt động xây dựng (nangluchdxd.gov.vn / Sở Xây dựng)</t>
+        </is>
+      </c>
+      <c r="C72" s="45" t="n"/>
+      <c r="D72" s="45" t="n"/>
+      <c r="E72" s="45" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="41" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="B73" s="41" t="inlineStr">
+        <is>
+          <t>Đơn vị đủ điều kiện thi công đường dây và trạm biến áp (điện lực tỉnh/EVN)</t>
+        </is>
+      </c>
+      <c r="C73" s="45" t="n"/>
+      <c r="D73" s="45" t="n"/>
+      <c r="E73" s="45" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="41" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="B74" s="41" t="inlineStr">
+        <is>
+          <t>Cổng thông tin quốc gia về đăng ký doanh nghiệp — theo mã ngành + địa bàn</t>
+        </is>
+      </c>
+      <c r="C74" s="45" t="n"/>
+      <c r="D74" s="45" t="n"/>
+      <c r="E74" s="45" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="41" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="B75" s="41" t="inlineStr">
+        <is>
+          <t>Sở Xây dựng / Sở Công Thương — công bố năng lực nhà thầu, giấy phép xây dựng</t>
+        </is>
+      </c>
+      <c r="C75" s="45" t="n"/>
+      <c r="D75" s="45" t="n"/>
+      <c r="E75" s="45" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="41" t="inlineStr">
+        <is>
+          <t>F6</t>
+        </is>
+      </c>
+      <c r="B76" s="41" t="inlineStr">
+        <is>
+          <t>Dự án ngược — chủ đầu tư, ban quản lý, báo chí công bố đơn vị thi công</t>
+        </is>
+      </c>
+      <c r="C76" s="45" t="n"/>
+      <c r="D76" s="45" t="n"/>
+      <c r="E76" s="45" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="41" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+      <c r="B77" s="41" t="inlineStr">
+        <is>
+          <t>Snowball — thầu phụ/liên danh nêu trong F1, F6; nhà thầu của CPO đối thủ</t>
+        </is>
+      </c>
+      <c r="C77" s="45" t="n"/>
+      <c r="D77" s="45" t="n"/>
+      <c r="E77" s="45" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="41" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
+      <c r="B78" s="41" t="inlineStr">
+        <is>
+          <t>Ngành lân cận — thầu điện, trạm biến áp, cơ điện M&amp;E, hạ tầng viễn thông</t>
+        </is>
+      </c>
+      <c r="C78" s="45" t="n"/>
+      <c r="D78" s="45" t="n"/>
+      <c r="E78" s="45" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="41" t="inlineStr">
+        <is>
+          <t>F9</t>
+        </is>
+      </c>
+      <c r="B79" s="41" t="inlineStr">
+        <is>
+          <t>Hiệp hội (VACC, hội nhà thầu/điện lực địa phương) — danh sách hội viên</t>
+        </is>
+      </c>
+      <c r="C79" s="45" t="n"/>
+      <c r="D79" s="45" t="n"/>
+      <c r="E79" s="45" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="41" t="inlineStr">
+        <is>
+          <t>F10</t>
+        </is>
+      </c>
+      <c r="B80" s="41" t="inlineStr">
+        <is>
+          <t>Trang đại lý ủy quyền của hãng thiết bị — dùng ngược để nhận diện Cấp 2</t>
+        </is>
+      </c>
+      <c r="C80" s="45" t="n"/>
+      <c r="D80" s="45" t="n"/>
+      <c r="E80" s="45" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="42" t="inlineStr">
+        <is>
+          <t>Bão hòa</t>
+        </is>
+      </c>
+      <c r="B81" s="41" t="inlineStr">
+        <is>
+          <t>Đạt khi hai khung liên tiếp không sinh MST mới VÀ F1–F5 đã quét hết. Chưa đạt thì ghi rõ chưa đạt và còn thiếu gì.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="42" t="inlineStr">
+        <is>
+          <t>Vùng mù còn lại</t>
+        </is>
+      </c>
+      <c r="B82" s="41" t="inlineStr">
+        <is>
+          <t>Ví dụ: đơn vị không có hiện diện web, gói thầu không công bố kết quả, tỉnh chưa quét, dữ liệu chứng chỉ chưa cập nhật.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="42" t="inlineStr">
+        <is>
+          <t>Tổng kết</t>
+        </is>
+      </c>
+      <c r="B83" s="41" t="inlineStr">
+        <is>
+          <t>Tổng số đơn vị | số Tổng thầu turnkey | số Nhóm A | số bị loại | bão hòa đạt/chưa.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A69:R69"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A46:R46"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>

</xml_diff>